<commit_message>
Add per-edge uplink communication model
</commit_message>
<xml_diff>
--- a/data/server_info.xlsx
+++ b/data/server_info.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,10 +451,15 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Uplink_Rate</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Latitude</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Longitude</t>
         </is>
@@ -476,9 +481,12 @@
         <v>0.02382984704172845</v>
       </c>
       <c r="E2" t="n">
+        <v>18</v>
+      </c>
+      <c r="F2" t="n">
         <v>-37.81517</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>144.97476</v>
       </c>
     </row>
@@ -498,9 +506,12 @@
         <v>0.01936962687103966</v>
       </c>
       <c r="E3" t="n">
+        <v>30</v>
+      </c>
+      <c r="F3" t="n">
         <v>-37.813175</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>144.952919</v>
       </c>
     </row>
@@ -520,9 +531,12 @@
         <v>0.01574422380749318</v>
       </c>
       <c r="E4" t="n">
+        <v>22</v>
+      </c>
+      <c r="F4" t="n">
         <v>-37.809081</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>144.96893</v>
       </c>
     </row>
@@ -542,9 +556,12 @@
         <v>0.01040210551357595</v>
       </c>
       <c r="E5" t="n">
+        <v>36</v>
+      </c>
+      <c r="F5" t="n">
         <v>-37.811022</v>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>144.959234</v>
       </c>
     </row>
@@ -564,9 +581,12 @@
         <v>0.008455148793793362</v>
       </c>
       <c r="E6" t="n">
+        <v>16</v>
+      </c>
+      <c r="F6" t="n">
         <v>-37.81679</v>
       </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>144.96918</v>
       </c>
     </row>
@@ -586,9 +606,12 @@
         <v>0.005586261409988603</v>
       </c>
       <c r="E7" t="n">
+        <v>28</v>
+      </c>
+      <c r="F7" t="n">
         <v>-37.818162</v>
       </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>144.959934</v>
       </c>
     </row>
@@ -608,9 +631,12 @@
         <v>0.004540683745308624</v>
       </c>
       <c r="E8" t="n">
+        <v>40</v>
+      </c>
+      <c r="F8" t="n">
         <v>-37.814395</v>
       </c>
-      <c r="F8" t="n">
+      <c r="G8" t="n">
         <v>144.963537</v>
       </c>
     </row>
@@ -630,9 +656,12 @@
         <v>0.003</v>
       </c>
       <c r="E9" t="n">
+        <v>24</v>
+      </c>
+      <c r="F9" t="n">
         <v>-37.82091</v>
       </c>
-      <c r="F9" t="n">
+      <c r="G9" t="n">
         <v>144.955155</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add fixed server transmission rates
</commit_message>
<xml_diff>
--- a/data/server_info.xlsx
+++ b/data/server_info.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,12 +449,17 @@
           <t>Base_Failure_Rate</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Transmission_Rate</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Latitude</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Longitude</t>
         </is>
@@ -476,9 +481,12 @@
         <v>0.003314111891641205</v>
       </c>
       <c r="E2" t="n">
+        <v>20</v>
+      </c>
+      <c r="F2" t="n">
         <v>-37.816356</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>144.962313</v>
       </c>
     </row>
@@ -498,9 +506,12 @@
         <v>0.004495975330962606</v>
       </c>
       <c r="E3" t="n">
+        <v>24</v>
+      </c>
+      <c r="F3" t="n">
         <v>-37.818071</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>144.957211</v>
       </c>
     </row>
@@ -520,9 +531,12 @@
         <v>0.001056376650416208</v>
       </c>
       <c r="E4" t="n">
+        <v>28</v>
+      </c>
+      <c r="F4" t="n">
         <v>-37.818202</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>144.954367</v>
       </c>
     </row>
@@ -542,9 +556,12 @@
         <v>0.004530516698436602</v>
       </c>
       <c r="E5" t="n">
+        <v>32</v>
+      </c>
+      <c r="F5" t="n">
         <v>-37.814225</v>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>144.971971</v>
       </c>
     </row>
@@ -564,9 +581,12 @@
         <v>0.002198760624193388</v>
       </c>
       <c r="E6" t="n">
+        <v>36</v>
+      </c>
+      <c r="F6" t="n">
         <v>-37.815975</v>
       </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>144.955905</v>
       </c>
     </row>
@@ -586,9 +606,12 @@
         <v>0.001402479155847763</v>
       </c>
       <c r="E7" t="n">
+        <v>40</v>
+      </c>
+      <c r="F7" t="n">
         <v>-37.815309</v>
       </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>144.969476</v>
       </c>
     </row>
@@ -608,9 +631,12 @@
         <v>0.00186812972709297</v>
       </c>
       <c r="E8" t="n">
+        <v>45</v>
+      </c>
+      <c r="F8" t="n">
         <v>-37.81208400000001</v>
       </c>
-      <c r="F8" t="n">
+      <c r="G8" t="n">
         <v>144.967997</v>
       </c>
     </row>
@@ -630,9 +656,12 @@
         <v>0.001704282643518897</v>
       </c>
       <c r="E9" t="n">
+        <v>50</v>
+      </c>
+      <c r="F9" t="n">
         <v>-37.814395</v>
       </c>
-      <c r="F9" t="n">
+      <c r="G9" t="n">
         <v>144.963537</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Freeze seeded profiles and record reproducible PPO baseline
</commit_message>
<xml_diff>
--- a/data/server_info.xlsx
+++ b/data/server_info.xlsx
@@ -449,7 +449,7 @@
           <t>Base_Failure_Rate</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Transmission_Rate</t>
         </is>
@@ -475,10 +475,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>10.46</v>
+        <v>10.6</v>
       </c>
       <c r="D2" t="n">
-        <v>0.003314111891641205</v>
+        <v>0.004133493529932761</v>
       </c>
       <c r="E2" t="n">
         <v>20</v>
@@ -500,10 +500,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>10.43</v>
+        <v>12.51</v>
       </c>
       <c r="D3" t="n">
-        <v>0.004495975330962606</v>
+        <v>0.003191245819401793</v>
       </c>
       <c r="E3" t="n">
         <v>24</v>
@@ -525,10 +525,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>12.28</v>
+        <v>12.56</v>
       </c>
       <c r="D4" t="n">
-        <v>0.001056376650416208</v>
+        <v>0.003922155969636815</v>
       </c>
       <c r="E4" t="n">
         <v>28</v>
@@ -550,10 +550,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>11.08</v>
+        <v>14.3</v>
       </c>
       <c r="D5" t="n">
-        <v>0.004530516698436602</v>
+        <v>0.004072461291876566</v>
       </c>
       <c r="E5" t="n">
         <v>32</v>
@@ -578,7 +578,7 @@
         <v>10.51</v>
       </c>
       <c r="D6" t="n">
-        <v>0.002198760624193388</v>
+        <v>0.004004103832634472</v>
       </c>
       <c r="E6" t="n">
         <v>36</v>
@@ -600,10 +600,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>11.66</v>
+        <v>11.12</v>
       </c>
       <c r="D7" t="n">
-        <v>0.001402479155847763</v>
+        <v>0.003346083385977</v>
       </c>
       <c r="E7" t="n">
         <v>40</v>
@@ -625,10 +625,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>10.24</v>
+        <v>13.01</v>
       </c>
       <c r="D8" t="n">
-        <v>0.00186812972709297</v>
+        <v>0.001959736317471708</v>
       </c>
       <c r="E8" t="n">
         <v>45</v>
@@ -650,10 +650,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>11.12</v>
+        <v>12.78</v>
       </c>
       <c r="D9" t="n">
-        <v>0.001704282643518897</v>
+        <v>0.003456817122719397</v>
       </c>
       <c r="E9" t="n">
         <v>50</v>

</xml_diff>

<commit_message>
Unify system parameters and reproducible train/evaluation profiles
</commit_message>
<xml_diff>
--- a/data/server_info.xlsx
+++ b/data/server_info.xlsx
@@ -475,13 +475,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>10.6</v>
+        <v>1656813293.530118</v>
       </c>
       <c r="D2" t="n">
-        <v>0.004133493529932761</v>
+        <v>0.004658194260187031</v>
       </c>
       <c r="E2" t="n">
-        <v>20</v>
+        <v>17.60938142345376</v>
       </c>
       <c r="F2" t="n">
         <v>-37.816356</v>
@@ -500,13 +500,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>12.51</v>
+        <v>2577350652.823907</v>
       </c>
       <c r="D3" t="n">
-        <v>0.003191245819401793</v>
+        <v>0.003316422013631598</v>
       </c>
       <c r="E3" t="n">
-        <v>24</v>
+        <v>26.93795996354849</v>
       </c>
       <c r="F3" t="n">
         <v>-37.818071</v>
@@ -525,13 +525,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>12.56</v>
+        <v>2888999728.276822</v>
       </c>
       <c r="D4" t="n">
-        <v>0.003922155969636815</v>
+        <v>0.004934879836802591</v>
       </c>
       <c r="E4" t="n">
-        <v>28</v>
+        <v>29.51990522250403</v>
       </c>
       <c r="F4" t="n">
         <v>-37.818202</v>
@@ -550,13 +550,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>14.3</v>
+        <v>2995733728.615859</v>
       </c>
       <c r="D5" t="n">
-        <v>0.004072461291876566</v>
+        <v>0.002439540755183242</v>
       </c>
       <c r="E5" t="n">
-        <v>32</v>
+        <v>28.72146783873085</v>
       </c>
       <c r="F5" t="n">
         <v>-37.814225</v>
@@ -575,13 +575,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>10.51</v>
+        <v>2876038204.791759</v>
       </c>
       <c r="D6" t="n">
-        <v>0.004004103832634472</v>
+        <v>0.001890892101121081</v>
       </c>
       <c r="E6" t="n">
-        <v>36</v>
+        <v>17.21600253706232</v>
       </c>
       <c r="F6" t="n">
         <v>-37.815975</v>
@@ -600,13 +600,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>11.12</v>
+        <v>1173005399.63119</v>
       </c>
       <c r="D7" t="n">
-        <v>0.003346083385977</v>
+        <v>0.002854266611664797</v>
       </c>
       <c r="E7" t="n">
-        <v>40</v>
+        <v>22.95926410853527</v>
       </c>
       <c r="F7" t="n">
         <v>-37.815309</v>
@@ -625,13 +625,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>13.01</v>
+        <v>1602970438.334235</v>
       </c>
       <c r="D8" t="n">
-        <v>0.001959736317471708</v>
+        <v>0.002595797927454248</v>
       </c>
       <c r="E8" t="n">
-        <v>45</v>
+        <v>29.71014280448686</v>
       </c>
       <c r="F8" t="n">
         <v>-37.81208400000001</v>
@@ -650,13 +650,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>12.78</v>
+        <v>1293731561.759833</v>
       </c>
       <c r="D9" t="n">
-        <v>0.003456817122719397</v>
+        <v>0.001991471355040274</v>
       </c>
       <c r="E9" t="n">
-        <v>50</v>
+        <v>20.9630893899643</v>
       </c>
       <c r="F9" t="n">
         <v>-37.814395</v>

</xml_diff>

<commit_message>
Unify simulator parameters and add PPO-Greedy latency experiments
</commit_message>
<xml_diff>
--- a/data/server_info.xlsx
+++ b/data/server_info.xlsx
@@ -475,13 +475,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1656813293.530118</v>
+        <v>1985219940.295177</v>
       </c>
       <c r="D2" t="n">
-        <v>0.004658194260187031</v>
+        <v>0.4658194260187031</v>
       </c>
       <c r="E2" t="n">
-        <v>17.60938142345376</v>
+        <v>10.70703606759032</v>
       </c>
       <c r="F2" t="n">
         <v>-37.816356</v>
@@ -500,13 +500,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2577350652.823907</v>
+        <v>3366025979.23586</v>
       </c>
       <c r="D3" t="n">
-        <v>0.003316422013631598</v>
+        <v>0.3316422013631598</v>
       </c>
       <c r="E3" t="n">
-        <v>26.93795996354849</v>
+        <v>17.70346997266137</v>
       </c>
       <c r="F3" t="n">
         <v>-37.818071</v>
@@ -525,13 +525,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2888999728.276822</v>
+        <v>3833499592.415233</v>
       </c>
       <c r="D4" t="n">
-        <v>0.004934879836802591</v>
+        <v>0.4934879836802591</v>
       </c>
       <c r="E4" t="n">
-        <v>29.51990522250403</v>
+        <v>19.63992891687802</v>
       </c>
       <c r="F4" t="n">
         <v>-37.818202</v>
@@ -550,13 +550,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2995733728.615859</v>
+        <v>3993600592.923788</v>
       </c>
       <c r="D5" t="n">
-        <v>0.002439540755183242</v>
+        <v>0.2439540755183242</v>
       </c>
       <c r="E5" t="n">
-        <v>28.72146783873085</v>
+        <v>19.04110087904814</v>
       </c>
       <c r="F5" t="n">
         <v>-37.814225</v>
@@ -575,13 +575,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2876038204.791759</v>
+        <v>3814057307.187637</v>
       </c>
       <c r="D6" t="n">
-        <v>0.001890892101121081</v>
+        <v>0.1890892101121081</v>
       </c>
       <c r="E6" t="n">
-        <v>17.21600253706232</v>
+        <v>10.41200190279674</v>
       </c>
       <c r="F6" t="n">
         <v>-37.815975</v>
@@ -600,13 +600,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1173005399.63119</v>
+        <v>1259508099.446785</v>
       </c>
       <c r="D7" t="n">
-        <v>0.002854266611664797</v>
+        <v>0.2854266611664797</v>
       </c>
       <c r="E7" t="n">
-        <v>22.95926410853527</v>
+        <v>14.71944808140145</v>
       </c>
       <c r="F7" t="n">
         <v>-37.815309</v>
@@ -625,13 +625,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1602970438.334235</v>
+        <v>1904455657.501352</v>
       </c>
       <c r="D8" t="n">
-        <v>0.002595797927454248</v>
+        <v>0.2595797927454248</v>
       </c>
       <c r="E8" t="n">
-        <v>29.71014280448686</v>
+        <v>19.78260710336515</v>
       </c>
       <c r="F8" t="n">
         <v>-37.81208400000001</v>
@@ -650,13 +650,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1293731561.759833</v>
+        <v>1440597342.639749</v>
       </c>
       <c r="D9" t="n">
-        <v>0.001991471355040274</v>
+        <v>0.1991471355040274</v>
       </c>
       <c r="E9" t="n">
-        <v>20.9630893899643</v>
+        <v>13.22231704247323</v>
       </c>
       <c r="F9" t="n">
         <v>-37.814395</v>

</xml_diff>

<commit_message>
Update workload profiles and simplify simulator metrics
</commit_message>
<xml_diff>
--- a/data/server_info.xlsx
+++ b/data/server_info.xlsx
@@ -475,13 +475,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1985219940.295177</v>
+        <v>2568159097.662151</v>
       </c>
       <c r="D2" t="n">
-        <v>0.4658194260187031</v>
+        <v>0.03308301897102782</v>
       </c>
       <c r="E2" t="n">
-        <v>10.70703606759032</v>
+        <v>5.666040131900441</v>
       </c>
       <c r="F2" t="n">
         <v>-37.816356</v>
@@ -500,13 +500,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>3366025979.23586</v>
+        <v>3600913332.374745</v>
       </c>
       <c r="D3" t="n">
-        <v>0.3316422013631598</v>
+        <v>0.02127919154129173</v>
       </c>
       <c r="E3" t="n">
-        <v>17.70346997266137</v>
+        <v>19.95671105762462</v>
       </c>
       <c r="F3" t="n">
         <v>-37.818071</v>
@@ -525,13 +525,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>3833499592.415233</v>
+        <v>1434115965.948121</v>
       </c>
       <c r="D4" t="n">
-        <v>0.4934879836802591</v>
+        <v>0.02188333508531468</v>
       </c>
       <c r="E4" t="n">
-        <v>19.63992891687802</v>
+        <v>6.335743713692551</v>
       </c>
       <c r="F4" t="n">
         <v>-37.818202</v>
@@ -550,13 +550,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>3993600592.923788</v>
+        <v>1285026219.968428</v>
       </c>
       <c r="D5" t="n">
-        <v>0.2439540755183242</v>
+        <v>0.04538185881754378</v>
       </c>
       <c r="E5" t="n">
-        <v>19.04110087904814</v>
+        <v>15.64732774690789</v>
       </c>
       <c r="F5" t="n">
         <v>-37.814225</v>
@@ -575,13 +575,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>3814057307.187637</v>
+        <v>1915630316.621437</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1890892101121081</v>
+        <v>0.03331816048323749</v>
       </c>
       <c r="E6" t="n">
-        <v>10.41200190279674</v>
+        <v>5.550983443135474</v>
       </c>
       <c r="F6" t="n">
         <v>-37.815975</v>
@@ -600,13 +600,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1259508099.446785</v>
+        <v>3632059326.788826</v>
       </c>
       <c r="D7" t="n">
-        <v>0.2854266611664797</v>
+        <v>0.04839714636394452</v>
       </c>
       <c r="E7" t="n">
-        <v>14.71944808140145</v>
+        <v>6.244974719187336</v>
       </c>
       <c r="F7" t="n">
         <v>-37.815309</v>
@@ -625,13 +625,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1904455657.501352</v>
+        <v>3294891766.923334</v>
       </c>
       <c r="D8" t="n">
-        <v>0.2595797927454248</v>
+        <v>0.02597211352937353</v>
       </c>
       <c r="E8" t="n">
-        <v>19.78260710336515</v>
+        <v>12.56351325798589</v>
       </c>
       <c r="F8" t="n">
         <v>-37.81208400000001</v>
@@ -650,13 +650,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1440597342.639749</v>
+        <v>2957805400.938731</v>
       </c>
       <c r="D9" t="n">
-        <v>0.1991471355040274</v>
+        <v>0.02662550585483387</v>
       </c>
       <c r="E9" t="n">
-        <v>13.22231704247323</v>
+        <v>13.51329234606641</v>
       </c>
       <c r="F9" t="n">
         <v>-37.814395</v>

</xml_diff>